<commit_message>
- Changed naming scheme to reduce confusion - Changed die pad numbering to match die diagrams (start with pad 0)
</commit_message>
<xml_diff>
--- a/docs/2026-05-18 Working out pin mapping.xlsx
+++ b/docs/2026-05-18 Working out pin mapping.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lauri\OneDrive\Firefly\Projects\BondTest72\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f9131ab26eb6539b/Firefly/Projects/BondTest72/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{930CE1AE-0B7B-40CB-9263-9D84E504AE9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="164" documentId="13_ncr:1_{930CE1AE-0B7B-40CB-9263-9D84E504AE9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13FB53D2-D81C-1649-98C3-137FD50317EE}"/>
   <bookViews>
-    <workbookView xWindow="4080" yWindow="1545" windowWidth="25125" windowHeight="18525" xr2:uid="{26C4B33B-203C-45C3-8015-FC1298DD10E7}"/>
+    <workbookView xWindow="17080" yWindow="820" windowWidth="17120" windowHeight="20260" activeTab="1" xr2:uid="{26C4B33B-203C-45C3-8015-FC1298DD10E7}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="1x1" sheetId="1" r:id="rId1"/>
+    <sheet name="1x0p5" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="79">
   <si>
     <t>Die</t>
   </si>
@@ -50,9 +51,6 @@
     <t>Pad number</t>
   </si>
   <si>
-    <t>BP number</t>
-  </si>
-  <si>
     <t>user_defined</t>
   </si>
   <si>
@@ -81,13 +79,211 @@
   </si>
   <si>
     <t>Tester ch</t>
+  </si>
+  <si>
+    <t>clk</t>
+  </si>
+  <si>
+    <t>rst_n</t>
+  </si>
+  <si>
+    <t>bidir_0</t>
+  </si>
+  <si>
+    <t>bidir_1</t>
+  </si>
+  <si>
+    <t>bidir_2</t>
+  </si>
+  <si>
+    <t>bidir_3</t>
+  </si>
+  <si>
+    <t>bidir_4</t>
+  </si>
+  <si>
+    <t>bidir_5</t>
+  </si>
+  <si>
+    <t>bidir_6</t>
+  </si>
+  <si>
+    <t>bidir_7</t>
+  </si>
+  <si>
+    <t>bidir_8</t>
+  </si>
+  <si>
+    <t>bidir_9</t>
+  </si>
+  <si>
+    <t>bidir_10</t>
+  </si>
+  <si>
+    <t>bidir_11</t>
+  </si>
+  <si>
+    <t>bidir_12</t>
+  </si>
+  <si>
+    <t>bidir_13</t>
+  </si>
+  <si>
+    <t>bidir_14</t>
+  </si>
+  <si>
+    <t>bidir_15</t>
+  </si>
+  <si>
+    <t>GND</t>
+  </si>
+  <si>
+    <t>VDD CORE</t>
+  </si>
+  <si>
+    <t>bidir_16</t>
+  </si>
+  <si>
+    <t>bidir_17</t>
+  </si>
+  <si>
+    <t>bidir_18</t>
+  </si>
+  <si>
+    <t>bidir_19</t>
+  </si>
+  <si>
+    <t>bidir_20</t>
+  </si>
+  <si>
+    <t>bidir_21</t>
+  </si>
+  <si>
+    <t>bidir_22</t>
+  </si>
+  <si>
+    <t>bidir_23</t>
+  </si>
+  <si>
+    <t>bidir_24</t>
+  </si>
+  <si>
+    <t>bidir_25</t>
+  </si>
+  <si>
+    <t>bidir_26</t>
+  </si>
+  <si>
+    <t>bidir_27</t>
+  </si>
+  <si>
+    <t>bidir_28</t>
+  </si>
+  <si>
+    <t>bidir_29</t>
+  </si>
+  <si>
+    <t>bidir_30</t>
+  </si>
+  <si>
+    <t>bidir_31</t>
+  </si>
+  <si>
+    <t>bidir_32</t>
+  </si>
+  <si>
+    <t>bidir_33</t>
+  </si>
+  <si>
+    <t>bidir_34</t>
+  </si>
+  <si>
+    <t>bidir_35</t>
+  </si>
+  <si>
+    <t>bidir_36</t>
+  </si>
+  <si>
+    <t>bidir_37</t>
+  </si>
+  <si>
+    <t>bidir_38</t>
+  </si>
+  <si>
+    <t>bidir_39</t>
+  </si>
+  <si>
+    <t>bidir_40</t>
+  </si>
+  <si>
+    <t>bidir_41</t>
+  </si>
+  <si>
+    <t>bidir_42</t>
+  </si>
+  <si>
+    <t>bidir_43</t>
+  </si>
+  <si>
+    <t>bidir_44</t>
+  </si>
+  <si>
+    <t>bidir_45</t>
+  </si>
+  <si>
+    <t>an_0</t>
+  </si>
+  <si>
+    <t>an_1</t>
+  </si>
+  <si>
+    <t>an_2</t>
+  </si>
+  <si>
+    <t>an_3</t>
+  </si>
+  <si>
+    <t>in_0</t>
+  </si>
+  <si>
+    <t>in_1</t>
+  </si>
+  <si>
+    <t>in_2</t>
+  </si>
+  <si>
+    <t>in_3</t>
+  </si>
+  <si>
+    <t>VDD IO 3</t>
+  </si>
+  <si>
+    <t>VDD CORE 1</t>
+  </si>
+  <si>
+    <t>PWR Aux 1</t>
+  </si>
+  <si>
+    <t>VDD IO 2</t>
+  </si>
+  <si>
+    <t>VDD IO 1</t>
+  </si>
+  <si>
+    <t>VDD IO 0</t>
+  </si>
+  <si>
+    <t>PWR Aux 0</t>
+  </si>
+  <si>
+    <t>Die pad</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -99,6 +295,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -148,27 +350,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -186,6 +385,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -506,69 +709,69 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1FA06EA-4DB4-46F8-AD15-2FDC3398CFA0}">
   <dimension ref="B2:G78"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.5703125" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" customWidth="1"/>
-    <col min="5" max="5" width="3.140625" customWidth="1"/>
-    <col min="6" max="6" width="11.85546875" customWidth="1"/>
-    <col min="7" max="7" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.5" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1640625" customWidth="1"/>
+    <col min="4" max="4" width="13.5" customWidth="1"/>
+    <col min="5" max="5" width="3.1640625" customWidth="1"/>
+    <col min="6" max="6" width="11.83203125" customWidth="1"/>
+    <col min="7" max="7" width="19.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
+    <row r="2" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="5"/>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B3" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="6"/>
+      <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3"/>
+      <c r="F3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B4" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="3"/>
+      <c r="F4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="3"/>
-    </row>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B3" s="4" t="s">
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B5">
         <v>0</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="6"/>
-      <c r="F3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B4" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E4" s="7"/>
-      <c r="F4" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B5">
-        <v>1</v>
-      </c>
       <c r="C5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D5">
         <v>8</v>
@@ -580,12 +783,12 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D6">
         <v>7</v>
@@ -597,12 +800,12 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D7">
         <v>6</v>
@@ -614,12 +817,12 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D8">
         <v>5</v>
@@ -631,12 +834,12 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D9">
         <v>4</v>
@@ -648,12 +851,12 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C10" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D10">
         <v>3</v>
@@ -665,12 +868,12 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B11">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D11">
         <v>2</v>
@@ -682,12 +885,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B12">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C12" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -699,20 +902,20 @@
         <v>69</v>
       </c>
     </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B13">
+        <v>8</v>
+      </c>
+      <c r="C13" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B14">
         <v>9</v>
       </c>
-      <c r="C13" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B14">
-        <v>10</v>
-      </c>
       <c r="C14" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D14">
         <v>70</v>
@@ -724,12 +927,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B15">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C15" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D15">
         <v>69</v>
@@ -741,12 +944,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B16">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C16" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D16">
         <v>68</v>
@@ -758,12 +961,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C17" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D17">
         <v>67</v>
@@ -775,12 +978,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C18" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D18">
         <v>66</v>
@@ -792,12 +995,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B19">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C19" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D19">
         <v>65</v>
@@ -809,12 +1012,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C20" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D20">
         <v>64</v>
@@ -826,12 +1029,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B21">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C21" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D21">
         <v>63</v>
@@ -843,12 +1046,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B22">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C22" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D22">
         <v>62</v>
@@ -860,12 +1063,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C23" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D23">
         <v>61</v>
@@ -877,12 +1080,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B24">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C24" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D24">
         <v>60</v>
@@ -894,12 +1097,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B25">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C25" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D25">
         <v>59</v>
@@ -911,12 +1114,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C26" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D26">
         <v>58</v>
@@ -928,12 +1131,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B27">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D27">
         <v>57</v>
@@ -945,12 +1148,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C28" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D28">
         <v>56</v>
@@ -962,12 +1165,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B29">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C29" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D29">
         <v>55</v>
@@ -979,12 +1182,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C30" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D30">
         <v>54</v>
@@ -996,12 +1199,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B31">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C31" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D31">
         <v>53</v>
@@ -1013,12 +1216,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C32" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D32">
         <v>52</v>
@@ -1030,12 +1233,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B33">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C33" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D33">
         <v>51</v>
@@ -1047,12 +1250,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B34">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C34" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D34">
         <v>50</v>
@@ -1064,12 +1267,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B35">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C35" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D35">
         <v>49</v>
@@ -1081,12 +1284,12 @@
         <v>21</v>
       </c>
     </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B36">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C36" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D36">
         <v>48</v>
@@ -1098,12 +1301,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B37">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C37" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D37">
         <v>47</v>
@@ -1115,20 +1318,20 @@
         <v>23</v>
       </c>
     </row>
-    <row r="38" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B38">
+        <v>33</v>
+      </c>
+      <c r="C38" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B39">
         <v>34</v>
       </c>
-      <c r="C38" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B39">
-        <v>35</v>
-      </c>
       <c r="C39" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D39">
         <v>46</v>
@@ -1140,12 +1343,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B40">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C40" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D40">
         <v>45</v>
@@ -1157,12 +1360,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="41" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B41">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C41" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D41">
         <v>44</v>
@@ -1174,12 +1377,12 @@
         <v>26</v>
       </c>
     </row>
-    <row r="42" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B42">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C42" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D42">
         <v>43</v>
@@ -1191,12 +1394,12 @@
         <v>27</v>
       </c>
     </row>
-    <row r="43" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B43">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C43" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D43">
         <v>42</v>
@@ -1208,12 +1411,12 @@
         <v>28</v>
       </c>
     </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B44">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C44" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D44">
         <v>41</v>
@@ -1225,12 +1428,12 @@
         <v>29</v>
       </c>
     </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B45">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C45" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D45">
         <v>40</v>
@@ -1242,12 +1445,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="46" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B46">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C46" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D46">
         <v>39</v>
@@ -1259,12 +1462,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B47">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C47" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D47">
         <v>38</v>
@@ -1276,12 +1479,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="48" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B48">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C48" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D48">
         <v>37</v>
@@ -1293,12 +1496,12 @@
         <v>33</v>
       </c>
     </row>
-    <row r="49" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B49">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C49" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D49">
         <v>36</v>
@@ -1310,20 +1513,20 @@
         <v>34</v>
       </c>
     </row>
-    <row r="50" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B50">
+        <v>45</v>
+      </c>
+      <c r="C50" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="51" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B51">
         <v>46</v>
       </c>
-      <c r="C50" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="51" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B51">
-        <v>47</v>
-      </c>
       <c r="C51" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D51">
         <v>35</v>
@@ -1335,12 +1538,12 @@
         <v>35</v>
       </c>
     </row>
-    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B52">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C52" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D52">
         <v>34</v>
@@ -1352,12 +1555,12 @@
         <v>36</v>
       </c>
     </row>
-    <row r="53" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B53">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C53" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D53">
         <v>33</v>
@@ -1369,12 +1572,12 @@
         <v>37</v>
       </c>
     </row>
-    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B54">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C54" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D54">
         <v>32</v>
@@ -1386,12 +1589,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="55" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B55">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C55" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D55">
         <v>31</v>
@@ -1403,12 +1606,12 @@
         <v>39</v>
       </c>
     </row>
-    <row r="56" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B56">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C56" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D56">
         <v>30</v>
@@ -1420,12 +1623,12 @@
         <v>40</v>
       </c>
     </row>
-    <row r="57" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B57">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C57" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D57">
         <v>29</v>
@@ -1437,12 +1640,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="58" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B58">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C58" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D58">
         <v>28</v>
@@ -1454,12 +1657,12 @@
         <v>42</v>
       </c>
     </row>
-    <row r="59" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B59">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C59" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D59">
         <v>27</v>
@@ -1471,12 +1674,12 @@
         <v>43</v>
       </c>
     </row>
-    <row r="60" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B60">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C60" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D60">
         <v>26</v>
@@ -1488,12 +1691,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="61" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B61">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C61" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D61">
         <v>25</v>
@@ -1505,12 +1708,12 @@
         <v>45</v>
       </c>
     </row>
-    <row r="62" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B62">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C62" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D62">
         <v>24</v>
@@ -1522,12 +1725,12 @@
         <v>46</v>
       </c>
     </row>
-    <row r="63" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B63">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C63" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D63">
         <v>23</v>
@@ -1539,12 +1742,12 @@
         <v>47</v>
       </c>
     </row>
-    <row r="64" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B64">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C64" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D64">
         <v>22</v>
@@ -1556,12 +1759,12 @@
         <v>48</v>
       </c>
     </row>
-    <row r="65" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B65">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C65" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D65">
         <v>21</v>
@@ -1573,12 +1776,12 @@
         <v>49</v>
       </c>
     </row>
-    <row r="66" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B66">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C66" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D66">
         <v>20</v>
@@ -1590,12 +1793,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="67" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B67">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C67" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D67">
         <v>18</v>
@@ -1607,12 +1810,12 @@
         <v>52</v>
       </c>
     </row>
-    <row r="68" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B68">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C68" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D68">
         <v>19</v>
@@ -1624,12 +1827,12 @@
         <v>51</v>
       </c>
     </row>
-    <row r="69" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B69">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C69" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D69">
         <v>17</v>
@@ -1641,12 +1844,12 @@
         <v>53</v>
       </c>
     </row>
-    <row r="70" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B70">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C70" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D70">
         <v>16</v>
@@ -1658,12 +1861,12 @@
         <v>54</v>
       </c>
     </row>
-    <row r="71" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B71">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C71" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D71">
         <v>15</v>
@@ -1675,12 +1878,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="72" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B72">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C72" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D72">
         <v>14</v>
@@ -1692,12 +1895,12 @@
         <v>56</v>
       </c>
     </row>
-    <row r="73" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B73">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C73" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D73">
         <v>13</v>
@@ -1709,12 +1912,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="74" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B74">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C74" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D74">
         <v>12</v>
@@ -1726,20 +1929,20 @@
         <v>58</v>
       </c>
     </row>
-    <row r="75" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B75">
+        <v>70</v>
+      </c>
+      <c r="C75" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="76" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B76">
         <v>71</v>
       </c>
-      <c r="C75" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="76" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B76">
-        <v>72</v>
-      </c>
       <c r="C76" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D76">
         <v>11</v>
@@ -1751,12 +1954,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="77" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B77">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C77" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D77">
         <v>10</v>
@@ -1768,12 +1971,12 @@
         <v>60</v>
       </c>
     </row>
-    <row r="78" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B78">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C78" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D78">
         <v>9</v>
@@ -1794,4 +1997,1422 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E169A227-6870-0446-B26D-9788D82698DC}">
+  <dimension ref="B2:G76"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="6.5" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1640625" customWidth="1"/>
+    <col min="4" max="4" width="13.5" customWidth="1"/>
+    <col min="5" max="5" width="3.1640625" customWidth="1"/>
+    <col min="6" max="6" width="11.83203125" customWidth="1"/>
+    <col min="7" max="7" width="19.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="5"/>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B3" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="6"/>
+      <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3"/>
+      <c r="F3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B4" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="3"/>
+      <c r="F4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5">
+        <v>8</v>
+      </c>
+      <c r="F5">
+        <f t="shared" ref="F5:F13" si="0">71-D5</f>
+        <v>63</v>
+      </c>
+      <c r="G5">
+        <f>F5-1</f>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6">
+        <v>7</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="0"/>
+        <v>64</v>
+      </c>
+      <c r="G6">
+        <f t="shared" ref="G6:G69" si="1">F6-1</f>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7">
+        <v>6</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>65</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="1"/>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8">
+        <v>5</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="0"/>
+        <v>66</v>
+      </c>
+      <c r="G8">
+        <f t="shared" si="1"/>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B9">
+        <v>4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9">
+        <v>10</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="0"/>
+        <v>61</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="1"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B10">
+        <v>5</v>
+      </c>
+      <c r="C10" t="s">
+        <v>72</v>
+      </c>
+      <c r="D10">
+        <v>11</v>
+      </c>
+      <c r="F10">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="1"/>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B11">
+        <v>6</v>
+      </c>
+      <c r="C11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11">
+        <v>4</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="0"/>
+        <v>67</v>
+      </c>
+      <c r="G11">
+        <f t="shared" si="1"/>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B12">
+        <v>7</v>
+      </c>
+      <c r="C12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="0"/>
+        <v>68</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="1"/>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B13">
+        <v>8</v>
+      </c>
+      <c r="C13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13">
+        <v>2</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="0"/>
+        <v>69</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="1"/>
+        <v>68</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B14">
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <f>71-D14</f>
+        <v>70</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="1"/>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B15">
+        <v>10</v>
+      </c>
+      <c r="C15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15">
+        <v>70</v>
+      </c>
+      <c r="F15">
+        <f>71-D15</f>
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B16">
+        <v>11</v>
+      </c>
+      <c r="C16" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16">
+        <v>69</v>
+      </c>
+      <c r="F16">
+        <f t="shared" ref="F16:F75" si="2">71-D16</f>
+        <v>2</v>
+      </c>
+      <c r="G16">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B17">
+        <v>12</v>
+      </c>
+      <c r="C17" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17">
+        <v>68</v>
+      </c>
+      <c r="F17">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="G17">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B18">
+        <v>13</v>
+      </c>
+      <c r="C18" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18">
+        <v>67</v>
+      </c>
+      <c r="F18">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="G18">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B19">
+        <v>14</v>
+      </c>
+      <c r="C19" t="s">
+        <v>25</v>
+      </c>
+      <c r="D19">
+        <v>66</v>
+      </c>
+      <c r="F19">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B20">
+        <v>15</v>
+      </c>
+      <c r="C20" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20">
+        <v>65</v>
+      </c>
+      <c r="F20">
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B21">
+        <v>16</v>
+      </c>
+      <c r="C21" t="s">
+        <v>27</v>
+      </c>
+      <c r="D21">
+        <v>64</v>
+      </c>
+      <c r="F21">
+        <f t="shared" si="2"/>
+        <v>7</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B22">
+        <v>17</v>
+      </c>
+      <c r="C22" t="s">
+        <v>28</v>
+      </c>
+      <c r="D22">
+        <v>63</v>
+      </c>
+      <c r="F22">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B23">
+        <v>18</v>
+      </c>
+      <c r="C23" t="s">
+        <v>4</v>
+      </c>
+      <c r="D23">
+        <v>61</v>
+      </c>
+      <c r="F23">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B24">
+        <v>19</v>
+      </c>
+      <c r="C24" t="s">
+        <v>76</v>
+      </c>
+      <c r="D24">
+        <v>62</v>
+      </c>
+      <c r="F24">
+        <f t="shared" si="2"/>
+        <v>9</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B25">
+        <v>20</v>
+      </c>
+      <c r="C25" t="s">
+        <v>29</v>
+      </c>
+      <c r="D25">
+        <v>60</v>
+      </c>
+      <c r="F25">
+        <f t="shared" si="2"/>
+        <v>11</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B26">
+        <v>21</v>
+      </c>
+      <c r="C26" t="s">
+        <v>30</v>
+      </c>
+      <c r="D26">
+        <v>59</v>
+      </c>
+      <c r="F26">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="1"/>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B27">
+        <v>22</v>
+      </c>
+      <c r="C27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D27">
+        <v>58</v>
+      </c>
+      <c r="F27">
+        <f t="shared" si="2"/>
+        <v>13</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="1"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B28">
+        <v>23</v>
+      </c>
+      <c r="C28" t="s">
+        <v>34</v>
+      </c>
+      <c r="D28">
+        <v>57</v>
+      </c>
+      <c r="F28">
+        <f t="shared" si="2"/>
+        <v>14</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="1"/>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B29">
+        <v>24</v>
+      </c>
+      <c r="C29" t="s">
+        <v>31</v>
+      </c>
+      <c r="D29">
+        <v>53</v>
+      </c>
+      <c r="F29">
+        <f t="shared" si="2"/>
+        <v>18</v>
+      </c>
+      <c r="G29">
+        <f t="shared" si="1"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B30">
+        <v>25</v>
+      </c>
+      <c r="C30" t="s">
+        <v>77</v>
+      </c>
+      <c r="D30">
+        <v>54</v>
+      </c>
+      <c r="F30">
+        <f t="shared" si="2"/>
+        <v>17</v>
+      </c>
+      <c r="G30">
+        <f t="shared" si="1"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B31">
+        <v>26</v>
+      </c>
+      <c r="C31" t="s">
+        <v>35</v>
+      </c>
+      <c r="D31">
+        <v>56</v>
+      </c>
+      <c r="F31">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+      <c r="G31">
+        <f t="shared" si="1"/>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B32">
+        <v>27</v>
+      </c>
+      <c r="C32" t="s">
+        <v>36</v>
+      </c>
+      <c r="D32">
+        <v>55</v>
+      </c>
+      <c r="F32">
+        <f t="shared" si="2"/>
+        <v>16</v>
+      </c>
+      <c r="G32">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B33">
+        <v>28</v>
+      </c>
+      <c r="C33" t="s">
+        <v>37</v>
+      </c>
+      <c r="D33">
+        <v>52</v>
+      </c>
+      <c r="F33">
+        <f t="shared" si="2"/>
+        <v>19</v>
+      </c>
+      <c r="G33">
+        <f t="shared" si="1"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B34">
+        <v>29</v>
+      </c>
+      <c r="C34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D34">
+        <v>51</v>
+      </c>
+      <c r="F34">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="G34">
+        <f t="shared" si="1"/>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="35" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B35">
+        <v>30</v>
+      </c>
+      <c r="C35" t="s">
+        <v>39</v>
+      </c>
+      <c r="D35">
+        <v>50</v>
+      </c>
+      <c r="F35">
+        <f t="shared" si="2"/>
+        <v>21</v>
+      </c>
+      <c r="G35">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="36" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B36">
+        <v>31</v>
+      </c>
+      <c r="C36" t="s">
+        <v>40</v>
+      </c>
+      <c r="D36">
+        <v>49</v>
+      </c>
+      <c r="F36">
+        <f t="shared" si="2"/>
+        <v>22</v>
+      </c>
+      <c r="G36">
+        <f t="shared" si="1"/>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="37" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B37">
+        <v>32</v>
+      </c>
+      <c r="C37" t="s">
+        <v>41</v>
+      </c>
+      <c r="D37">
+        <v>48</v>
+      </c>
+      <c r="F37">
+        <f t="shared" si="2"/>
+        <v>23</v>
+      </c>
+      <c r="G37">
+        <f t="shared" si="1"/>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="38" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B38">
+        <v>33</v>
+      </c>
+      <c r="C38" t="s">
+        <v>42</v>
+      </c>
+      <c r="D38">
+        <v>47</v>
+      </c>
+      <c r="F38">
+        <f t="shared" si="2"/>
+        <v>24</v>
+      </c>
+      <c r="G38">
+        <f t="shared" si="1"/>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="39" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B39">
+        <v>34</v>
+      </c>
+      <c r="C39" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="40" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B40">
+        <v>35</v>
+      </c>
+      <c r="C40" t="s">
+        <v>75</v>
+      </c>
+      <c r="D40">
+        <v>44</v>
+      </c>
+      <c r="F40">
+        <f t="shared" si="2"/>
+        <v>27</v>
+      </c>
+      <c r="G40">
+        <f t="shared" si="1"/>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B41">
+        <v>36</v>
+      </c>
+      <c r="C41" t="s">
+        <v>43</v>
+      </c>
+      <c r="D41">
+        <v>43</v>
+      </c>
+      <c r="F41">
+        <f t="shared" si="2"/>
+        <v>28</v>
+      </c>
+      <c r="G41">
+        <f t="shared" si="1"/>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="42" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B42">
+        <v>37</v>
+      </c>
+      <c r="C42" t="s">
+        <v>44</v>
+      </c>
+      <c r="D42">
+        <v>42</v>
+      </c>
+      <c r="F42">
+        <f t="shared" si="2"/>
+        <v>29</v>
+      </c>
+      <c r="G42">
+        <f t="shared" si="1"/>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="43" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B43">
+        <v>38</v>
+      </c>
+      <c r="C43" t="s">
+        <v>45</v>
+      </c>
+      <c r="D43">
+        <v>41</v>
+      </c>
+      <c r="F43">
+        <f t="shared" si="2"/>
+        <v>30</v>
+      </c>
+      <c r="G43">
+        <f t="shared" si="1"/>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="44" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B44">
+        <v>39</v>
+      </c>
+      <c r="C44" t="s">
+        <v>46</v>
+      </c>
+      <c r="D44">
+        <v>40</v>
+      </c>
+      <c r="F44">
+        <f t="shared" si="2"/>
+        <v>31</v>
+      </c>
+      <c r="G44">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="45" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B45">
+        <v>40</v>
+      </c>
+      <c r="C45" t="s">
+        <v>32</v>
+      </c>
+      <c r="D45">
+        <v>46</v>
+      </c>
+      <c r="F45">
+        <f t="shared" si="2"/>
+        <v>25</v>
+      </c>
+      <c r="G45">
+        <f t="shared" si="1"/>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="46" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B46">
+        <v>41</v>
+      </c>
+      <c r="C46" t="s">
+        <v>31</v>
+      </c>
+      <c r="D46">
+        <v>45</v>
+      </c>
+      <c r="F46">
+        <f t="shared" si="2"/>
+        <v>26</v>
+      </c>
+      <c r="G46">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="47" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B47">
+        <v>42</v>
+      </c>
+      <c r="C47" t="s">
+        <v>47</v>
+      </c>
+      <c r="D47">
+        <v>39</v>
+      </c>
+      <c r="F47">
+        <f t="shared" si="2"/>
+        <v>32</v>
+      </c>
+      <c r="G47">
+        <f t="shared" si="1"/>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="48" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B48">
+        <v>43</v>
+      </c>
+      <c r="C48" t="s">
+        <v>48</v>
+      </c>
+      <c r="D48">
+        <v>38</v>
+      </c>
+      <c r="F48">
+        <f t="shared" si="2"/>
+        <v>33</v>
+      </c>
+      <c r="G48">
+        <f t="shared" si="1"/>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="49" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B49">
+        <v>44</v>
+      </c>
+      <c r="C49" t="s">
+        <v>49</v>
+      </c>
+      <c r="D49">
+        <v>37</v>
+      </c>
+      <c r="F49">
+        <f t="shared" si="2"/>
+        <v>34</v>
+      </c>
+      <c r="G49">
+        <f t="shared" si="1"/>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="50" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B50">
+        <v>45</v>
+      </c>
+      <c r="C50" t="s">
+        <v>50</v>
+      </c>
+      <c r="D50">
+        <v>36</v>
+      </c>
+      <c r="F50">
+        <f t="shared" si="2"/>
+        <v>35</v>
+      </c>
+      <c r="G50">
+        <f t="shared" si="1"/>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="51" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B51">
+        <v>46</v>
+      </c>
+      <c r="C51" t="s">
+        <v>51</v>
+      </c>
+      <c r="D51">
+        <v>35</v>
+      </c>
+      <c r="F51">
+        <f t="shared" si="2"/>
+        <v>36</v>
+      </c>
+      <c r="G51">
+        <f t="shared" si="1"/>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="52" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B52">
+        <v>47</v>
+      </c>
+      <c r="C52" t="s">
+        <v>52</v>
+      </c>
+      <c r="D52">
+        <v>34</v>
+      </c>
+      <c r="F52">
+        <f t="shared" si="2"/>
+        <v>37</v>
+      </c>
+      <c r="G52">
+        <f t="shared" si="1"/>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="53" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B53">
+        <v>48</v>
+      </c>
+      <c r="C53" t="s">
+        <v>53</v>
+      </c>
+      <c r="D53">
+        <v>33</v>
+      </c>
+      <c r="F53">
+        <f t="shared" si="2"/>
+        <v>38</v>
+      </c>
+      <c r="G53">
+        <f t="shared" si="1"/>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="54" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B54">
+        <v>49</v>
+      </c>
+      <c r="C54" t="s">
+        <v>54</v>
+      </c>
+      <c r="D54">
+        <v>32</v>
+      </c>
+      <c r="F54">
+        <f t="shared" si="2"/>
+        <v>39</v>
+      </c>
+      <c r="G54">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="55" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B55">
+        <v>50</v>
+      </c>
+      <c r="C55" t="s">
+        <v>55</v>
+      </c>
+      <c r="D55">
+        <v>31</v>
+      </c>
+      <c r="F55">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
+      <c r="G55">
+        <f t="shared" si="1"/>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="56" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B56">
+        <v>51</v>
+      </c>
+      <c r="C56" t="s">
+        <v>56</v>
+      </c>
+      <c r="D56">
+        <v>30</v>
+      </c>
+      <c r="F56">
+        <f t="shared" si="2"/>
+        <v>41</v>
+      </c>
+      <c r="G56">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="57" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B57">
+        <v>52</v>
+      </c>
+      <c r="C57" t="s">
+        <v>57</v>
+      </c>
+      <c r="D57">
+        <v>29</v>
+      </c>
+      <c r="F57">
+        <f t="shared" si="2"/>
+        <v>42</v>
+      </c>
+      <c r="G57">
+        <f t="shared" si="1"/>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="58" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B58">
+        <v>53</v>
+      </c>
+      <c r="C58" t="s">
+        <v>58</v>
+      </c>
+      <c r="D58">
+        <v>28</v>
+      </c>
+      <c r="F58">
+        <f t="shared" si="2"/>
+        <v>43</v>
+      </c>
+      <c r="G58">
+        <f t="shared" si="1"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="59" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B59">
+        <v>54</v>
+      </c>
+      <c r="C59" t="s">
+        <v>74</v>
+      </c>
+      <c r="D59">
+        <v>24</v>
+      </c>
+      <c r="F59">
+        <f t="shared" si="2"/>
+        <v>47</v>
+      </c>
+      <c r="G59">
+        <f t="shared" si="1"/>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="60" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B60">
+        <v>55</v>
+      </c>
+      <c r="C60" t="s">
+        <v>31</v>
+      </c>
+      <c r="D60">
+        <v>25</v>
+      </c>
+      <c r="F60">
+        <f t="shared" si="2"/>
+        <v>46</v>
+      </c>
+      <c r="G60">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="61" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B61">
+        <v>56</v>
+      </c>
+      <c r="C61" t="s">
+        <v>59</v>
+      </c>
+      <c r="D61">
+        <v>27</v>
+      </c>
+      <c r="F61">
+        <f t="shared" si="2"/>
+        <v>44</v>
+      </c>
+      <c r="G61">
+        <f t="shared" si="1"/>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="62" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B62">
+        <v>57</v>
+      </c>
+      <c r="C62" t="s">
+        <v>60</v>
+      </c>
+      <c r="D62">
+        <v>26</v>
+      </c>
+      <c r="F62">
+        <f t="shared" si="2"/>
+        <v>45</v>
+      </c>
+      <c r="G62">
+        <f t="shared" si="1"/>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="63" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B63">
+        <v>58</v>
+      </c>
+      <c r="C63" t="s">
+        <v>61</v>
+      </c>
+      <c r="D63">
+        <v>23</v>
+      </c>
+      <c r="F63">
+        <f t="shared" si="2"/>
+        <v>48</v>
+      </c>
+      <c r="G63">
+        <f t="shared" si="1"/>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="64" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B64">
+        <v>59</v>
+      </c>
+      <c r="C64" t="s">
+        <v>62</v>
+      </c>
+      <c r="D64">
+        <v>22</v>
+      </c>
+      <c r="F64">
+        <f t="shared" si="2"/>
+        <v>49</v>
+      </c>
+      <c r="G64">
+        <f t="shared" si="1"/>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="65" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B65">
+        <v>60</v>
+      </c>
+      <c r="C65" t="s">
+        <v>73</v>
+      </c>
+      <c r="D65">
+        <v>19</v>
+      </c>
+      <c r="F65">
+        <f t="shared" si="2"/>
+        <v>52</v>
+      </c>
+      <c r="G65">
+        <f t="shared" si="1"/>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="66" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B66">
+        <v>61</v>
+      </c>
+      <c r="C66" t="s">
+        <v>31</v>
+      </c>
+      <c r="D66">
+        <v>18</v>
+      </c>
+      <c r="F66">
+        <f t="shared" si="2"/>
+        <v>53</v>
+      </c>
+      <c r="G66">
+        <f t="shared" si="1"/>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="67" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B67">
+        <v>62</v>
+      </c>
+      <c r="C67" t="s">
+        <v>63</v>
+      </c>
+      <c r="D67">
+        <v>21</v>
+      </c>
+      <c r="F67">
+        <f t="shared" si="2"/>
+        <v>50</v>
+      </c>
+      <c r="G67">
+        <f t="shared" si="1"/>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="68" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B68">
+        <v>63</v>
+      </c>
+      <c r="C68" t="s">
+        <v>64</v>
+      </c>
+      <c r="D68">
+        <v>20</v>
+      </c>
+      <c r="F68">
+        <f t="shared" si="2"/>
+        <v>51</v>
+      </c>
+      <c r="G68">
+        <f t="shared" si="1"/>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="69" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B69">
+        <v>64</v>
+      </c>
+      <c r="C69" t="s">
+        <v>65</v>
+      </c>
+      <c r="D69">
+        <v>17</v>
+      </c>
+      <c r="F69">
+        <f t="shared" si="2"/>
+        <v>54</v>
+      </c>
+      <c r="G69">
+        <f t="shared" si="1"/>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="70" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B70">
+        <v>65</v>
+      </c>
+      <c r="C70" t="s">
+        <v>66</v>
+      </c>
+      <c r="D70">
+        <v>16</v>
+      </c>
+      <c r="F70">
+        <f t="shared" si="2"/>
+        <v>55</v>
+      </c>
+      <c r="G70">
+        <f t="shared" ref="G70:G75" si="3">F70-1</f>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="71" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B71">
+        <v>66</v>
+      </c>
+      <c r="C71" t="s">
+        <v>67</v>
+      </c>
+      <c r="D71">
+        <v>12</v>
+      </c>
+      <c r="F71">
+        <f t="shared" si="2"/>
+        <v>59</v>
+      </c>
+      <c r="G71">
+        <f t="shared" si="3"/>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="72" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B72">
+        <v>67</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>13</v>
+      </c>
+      <c r="F72">
+        <f t="shared" si="2"/>
+        <v>58</v>
+      </c>
+      <c r="G72">
+        <f t="shared" si="3"/>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="73" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B73">
+        <v>68</v>
+      </c>
+      <c r="C73" t="s">
+        <v>69</v>
+      </c>
+      <c r="D73">
+        <v>14</v>
+      </c>
+      <c r="F73">
+        <f t="shared" si="2"/>
+        <v>57</v>
+      </c>
+      <c r="G73">
+        <f t="shared" si="3"/>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="74" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B74">
+        <v>69</v>
+      </c>
+      <c r="C74" t="s">
+        <v>70</v>
+      </c>
+      <c r="D74">
+        <v>15</v>
+      </c>
+      <c r="F74">
+        <f t="shared" si="2"/>
+        <v>56</v>
+      </c>
+      <c r="G74">
+        <f t="shared" si="3"/>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="75" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B75">
+        <v>70</v>
+      </c>
+      <c r="C75" t="s">
+        <v>71</v>
+      </c>
+      <c r="D75">
+        <v>9</v>
+      </c>
+      <c r="F75">
+        <f t="shared" si="2"/>
+        <v>62</v>
+      </c>
+      <c r="G75">
+        <f t="shared" si="3"/>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="76" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B76">
+        <v>71</v>
+      </c>
+      <c r="C76" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B3:C3"/>
+  </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>